<commit_message>
Dodanie raportu końcowego testów oraz modyfikacja dokumentacji
</commit_message>
<xml_diff>
--- a/test-documentation/AutomationExercise_TestCases.xlsx
+++ b/test-documentation/AutomationExercise_TestCases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laptop\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laptop\Desktop\programowanie\Projekty\Projekty Git Repo\AutomationExercise-Playwright\test-documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1FA651-9C27-4C13-8CE9-5FEE7DAAC94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14986B78-E047-49F1-8C52-8273F1BF776E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="312">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -140,29 +140,6 @@
     <t>Pierwszy produkt zawiera wszystkie wymagane pola danych i spełnia podstawową walidację struktury odpowiedzi.</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">API zwróciło kod 404 oraz komunikat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>User not found!</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
     <t>1. Wysłać request POST tworzący konto użytkownika.                                                2. Zweryfikować możliwość logowania utworzonym kontem.                                  3. Wysłać request PUT aktualizujący dane użytkownika.                                                4. Pobrać szczegóły użytkownika po adresie email.                                                            5. Zweryfikować poprawność zaktualizowanych danych.                           6. Wysłać request DELETE usuwający konto.</t>
   </si>
   <si>
@@ -241,52 +218,6 @@
     <t>1. Przejść na podstronę „Products”.                       2. Najechać na wybrany produkt.                            3. Kliknąć „Add to cart”.                                             4. Zweryfikować modal potwierdzający.                  5. Przejść do widoku koszyka.</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Produkt powinien zostać dodany do koszyka z ilością równą </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Produkt został poprawnie dodany do koszyka, a ilość widoczna w tabeli koszyka wynosi </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
     <t>CART_005</t>
   </si>
   <si>
@@ -470,9 +401,6 @@
     <t>Zamówienie zostało potwierdzone, a aplikacja wyświetliła komunikat potwierdzający.</t>
   </si>
   <si>
-    <t>Positive / E2E</t>
-  </si>
-  <si>
     <t>PAY_008</t>
   </si>
   <si>
@@ -483,9 +411,6 @@
   </si>
   <si>
     <t>Aplikacja zaakceptowała niepoprawne dane i potwierdziła zamówienie.</t>
-  </si>
-  <si>
-    <t>Negative / Validation</t>
   </si>
   <si>
     <t>Known Bug</t>
@@ -624,55 +549,6 @@
     <t>Plik został poprawnie dodany, formularz został wysłany, a komunikat sukcesu został wyświetlony.</t>
   </si>
   <si>
-    <t>Positive / Upload</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Formularz nie powinien zostać wysłany, a komunikat walidacyjny powinien wskazywać brak znaku </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>@</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Formularz został zablokowany, a komunikat walidacyjny zawiera informację o wymaganym znaku </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>@</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
     <t>1. Przejść do formularza kontaktowego.     2. Zweryfikować widoczność pól: Name, Email, Subject, Message.                              3. Zweryfikować widoczność przycisku wyboru pliku.                                                  4. Zweryfikować widoczność przycisku Submit.</t>
   </si>
   <si>
@@ -682,29 +558,6 @@
     <t>1. Uzupełnić pola Name, Email, Subject oraz Message poprawnymi danymi.             2. Kliknąć Submit.                                               3. Zaakceptować okno dialogowe.                 4. Zweryfikować komunikat sukcesu.</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">1. Wpisać w pole Email wartość bez znaku </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>@</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.                                                                    2. Kliknąć Submit.                                         3. Sprawdzić komunikat walidacyjny pola Email.</t>
-    </r>
-  </si>
-  <si>
     <t>1. Uzupełnić tylko pole Email.                        2. Kliknąć Submit.                                          3. Zaakceptować okno dialogowe.              4. Zweryfikować, że komunikat sukcesu nie powinien się pojawić.</t>
   </si>
   <si>
@@ -780,29 +633,6 @@
     <t>1. Pozostawić pole email puste.                    2. Wpisać hasło.                                             3. Kliknąć Login.                                            4. Sprawdzić komunikat walidacyjny pola email.</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">1. Wpisać email bez znaku </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>@</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.                         2. Wpisać hasło.                                             3. Kliknąć Login.                                            4. Sprawdzić komunikat walidacyjny pola email.</t>
-    </r>
-  </si>
-  <si>
     <t>NAV_001</t>
   </si>
   <si>
@@ -912,9 +742,6 @@
   </si>
   <si>
     <t>Dla testowanych kategorii aplikacja wyświetla odpowiednie nagłówki oraz produkty przypisane do wybranych kategorii.</t>
-  </si>
-  <si>
-    <t>Positive / Data Driven</t>
   </si>
   <si>
     <t>1. Przejść na podstronę produktów.           2. Zweryfikować widoczność nagłówka „All Products”.                                                     3. Zweryfikować widoczność sekcji „Category”.                                                    4. Zweryfikować widoczność sekcji „Brands”.</t>
@@ -1199,6 +1026,12 @@
   </si>
   <si>
     <t xml:space="preserve">Negative </t>
+  </si>
+  <si>
+    <t>nameCard: Test User,
+numberCard: ABCD@@@@,
+cvcCard: ABC ,    monthCard: 99,
+yearCard: 2020,</t>
   </si>
 </sst>
 </file>
@@ -1553,12 +1386,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="13.5546875" style="1" customWidth="1"/>
     <col min="2" max="5" width="25.77734375" style="1"/>
-    <col min="6" max="6" width="40.77734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="38.6640625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="25.77734375" style="1"/>
   </cols>
   <sheetData>
@@ -1570,10 +1403,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>279</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>290</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>2</v>
@@ -1602,16 +1435,16 @@
         <v>9</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>11</v>
@@ -1620,7 +1453,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>13</v>
@@ -1634,16 +1467,16 @@
         <v>15</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>280</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>291</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>17</v>
@@ -1666,16 +1499,16 @@
         <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>22</v>
@@ -1698,16 +1531,16 @@
         <v>25</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>27</v>
@@ -1730,16 +1563,16 @@
         <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>32</v>
@@ -1748,7 +1581,7 @@
         <v>33</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>13</v>
@@ -1756,28 +1589,28 @@
     </row>
     <row r="7" spans="1:10" ht="93.6">
       <c r="A7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>29</v>
@@ -1788,28 +1621,28 @@
     </row>
     <row r="8" spans="1:10" ht="109.2">
       <c r="A8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>29</v>
@@ -1818,30 +1651,30 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="109.2">
+    <row r="9" spans="1:10" ht="124.8">
       <c r="A9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>29</v>
@@ -1852,28 +1685,28 @@
     </row>
     <row r="10" spans="1:10" ht="78">
       <c r="A10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>29</v>
@@ -1884,28 +1717,28 @@
     </row>
     <row r="11" spans="1:10" ht="93.6">
       <c r="A11" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>29</v>
@@ -1916,28 +1749,28 @@
     </row>
     <row r="12" spans="1:10" ht="78">
       <c r="A12" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>69</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>29</v>
@@ -1948,28 +1781,28 @@
     </row>
     <row r="13" spans="1:10" ht="78">
       <c r="A13" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>29</v>
@@ -1980,28 +1813,28 @@
     </row>
     <row r="14" spans="1:10" ht="109.2">
       <c r="A14" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>29</v>
@@ -2012,28 +1845,28 @@
     </row>
     <row r="15" spans="1:10" ht="109.2">
       <c r="A15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>29</v>
@@ -2044,31 +1877,31 @@
     </row>
     <row r="16" spans="1:10" ht="78">
       <c r="A16" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="I16" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>13</v>
@@ -2076,28 +1909,28 @@
     </row>
     <row r="17" spans="1:10" ht="78">
       <c r="A17" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>98</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>19</v>
@@ -2108,28 +1941,28 @@
     </row>
     <row r="18" spans="1:10" ht="78">
       <c r="A18" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>102</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>19</v>
@@ -2140,28 +1973,28 @@
     </row>
     <row r="19" spans="1:10" ht="78">
       <c r="A19" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="H19" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>106</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>19</v>
@@ -2172,28 +2005,28 @@
     </row>
     <row r="20" spans="1:10" ht="78">
       <c r="A20" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>107</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>110</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>19</v>
@@ -2204,28 +2037,28 @@
     </row>
     <row r="21" spans="1:10" ht="93.6">
       <c r="A21" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>119</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>19</v>
@@ -2236,95 +2069,95 @@
     </row>
     <row r="22" spans="1:10" ht="93.6">
       <c r="A22" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="E22" s="3" t="s">
+      <c r="I22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="124.8">
+      <c r="A23" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="G22" s="3" t="s">
+      <c r="B23" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="F23" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G23" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="I22" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="109.2">
-      <c r="A23" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>127</v>
-      </c>
       <c r="H23" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>19</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="140.4">
       <c r="A24" s="3" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>13</v>
@@ -2332,31 +2165,31 @@
     </row>
     <row r="25" spans="1:10" ht="109.2">
       <c r="A25" s="3" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>13</v>
@@ -2364,28 +2197,28 @@
     </row>
     <row r="26" spans="1:10" ht="93.6">
       <c r="A26" s="3" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>145</v>
-      </c>
       <c r="F26" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>19</v>
@@ -2396,28 +2229,28 @@
     </row>
     <row r="27" spans="1:10" ht="78">
       <c r="A27" s="3" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>29</v>
@@ -2428,28 +2261,28 @@
     </row>
     <row r="28" spans="1:10" ht="78">
       <c r="A28" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>19</v>
@@ -2460,60 +2293,60 @@
     </row>
     <row r="29" spans="1:10" ht="78">
       <c r="A29" s="3" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="109.2">
       <c r="A30" s="3" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>29</v>
@@ -2524,28 +2357,28 @@
     </row>
     <row r="31" spans="1:10" ht="93.6">
       <c r="A31" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>19</v>
@@ -2556,28 +2389,28 @@
     </row>
     <row r="32" spans="1:10" ht="78">
       <c r="A32" s="3" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>29</v>
@@ -2588,28 +2421,28 @@
     </row>
     <row r="33" spans="1:10" ht="78">
       <c r="A33" s="3" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>181</v>
-      </c>
       <c r="F33" s="3" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>19</v>
@@ -2620,28 +2453,28 @@
     </row>
     <row r="34" spans="1:10" ht="78">
       <c r="A34" s="3" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="I34" s="3" t="s">
         <v>19</v>
@@ -2652,28 +2485,28 @@
     </row>
     <row r="35" spans="1:10" ht="78">
       <c r="A35" s="3" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>19</v>
@@ -2684,28 +2517,28 @@
     </row>
     <row r="36" spans="1:10" ht="78">
       <c r="A36" s="3" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>29</v>
@@ -2716,28 +2549,28 @@
     </row>
     <row r="37" spans="1:10" ht="109.2">
       <c r="A37" s="3" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="I37" s="3" t="s">
         <v>29</v>
@@ -2748,28 +2581,28 @@
     </row>
     <row r="38" spans="1:10" ht="78">
       <c r="A38" s="3" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="G38" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>206</v>
-      </c>
       <c r="H38" s="3" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>29</v>
@@ -2780,28 +2613,28 @@
     </row>
     <row r="39" spans="1:10" ht="93.6">
       <c r="A39" s="3" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>29</v>
@@ -2812,28 +2645,28 @@
     </row>
     <row r="40" spans="1:10" ht="93.6">
       <c r="A40" s="3" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>29</v>
@@ -2844,28 +2677,28 @@
     </row>
     <row r="41" spans="1:10" ht="109.2">
       <c r="A41" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B41" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>233</v>
-      </c>
       <c r="G41" s="3" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="I41" s="3" t="s">
         <v>29</v>
@@ -2876,31 +2709,31 @@
     </row>
     <row r="42" spans="1:10" ht="109.2">
       <c r="A42" s="3" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J42" s="3" t="s">
         <v>13</v>
@@ -2908,28 +2741,28 @@
     </row>
     <row r="43" spans="1:10" ht="109.2">
       <c r="A43" s="3" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>29</v>
@@ -2940,31 +2773,31 @@
     </row>
     <row r="44" spans="1:10" ht="109.2">
       <c r="A44" s="3" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J44" s="3" t="s">
         <v>13</v>
@@ -2972,28 +2805,28 @@
     </row>
     <row r="45" spans="1:10" ht="93.6">
       <c r="A45" s="3" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>19</v>
@@ -3004,92 +2837,92 @@
     </row>
     <row r="46" spans="1:10" ht="109.2">
       <c r="A46" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="F46" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="B46" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>257</v>
-      </c>
       <c r="G46" s="3" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>19</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="109.2">
       <c r="A47" s="3" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="109.2">
       <c r="A48" s="3" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="I48" s="3" t="s">
         <v>19</v>
@@ -3100,28 +2933,28 @@
     </row>
     <row r="49" spans="1:10" ht="78">
       <c r="A49" s="3" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="F49" s="3" t="s">
-        <v>276</v>
-      </c>
       <c r="G49" s="3" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="I49" s="3" t="s">
         <v>19</v>
@@ -3132,28 +2965,28 @@
     </row>
     <row r="50" spans="1:10" ht="78">
       <c r="A50" s="3" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>19</v>
@@ -3164,28 +2997,28 @@
     </row>
     <row r="51" spans="1:10" ht="124.8">
       <c r="A51" s="3" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>29</v>

</xml_diff>